<commit_message>
fix(export): Cloud Cowboy logo top-left on every exported sheet
The proforma template already carried the brand palette and the logo image,
and the exceljs round-trip preserves both — but the Proforma and Monthly Cash
Flow sheets anchored the logo at the bottom (rows 98 / 29) instead of the
top-left like the other five sheets.

Patched the template so all seven sheets place the logo in a tall top-left
row 1, matching the Events/Orgs/Capital/Seasonality/Notes sheets (raised the
Proforma row-1 height to 46 to hold it). Image, drawings, and brand colors all
survive the export round-trip.

Added export-test assertions: the logo image is present, there are seven
drawings, and every sheet's logo is anchored in the top row.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/proforma-template.xlsx
+++ b/public/proforma-template.xlsx
@@ -3042,15 +3042,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>98</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>50800</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>513000</xdr:colOff>
-      <xdr:row>111</xdr:row>
-      <xdr:rowOff>42840</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1669720</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>488620</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3163,15 +3163,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>50800</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>581760</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>21960</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1669720</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>488620</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3676,7 +3676,7 @@
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
     </row>
     <row r="2" spans="1:10" ht="19" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
fix(export): correct Proforma logo placement (match the other sheets)
The previous patch targeted the wrong anchor: the Proforma sheet's drawing
holds two charts plus the logo, and the string-replace moved a chart to the
top-left instead of the logo — leaving the logo warped/oversized and
overlapping the title row.

This time patch only the logo <xdr:pic> anchor so it sits fully inside a tall
top-left row 1 (height 46), byte-identical to the Events/Orgs/Capital/
Seasonality/Notes sheets, and verified to survive the exceljs export
round-trip unchanged. Charts in the template are left untouched.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/proforma-template.xlsx
+++ b/public/proforma-template.xlsx
@@ -3042,15 +3042,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>50800</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>98</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1669720</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>488620</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>513000</xdr:colOff>
+      <xdr:row>111</xdr:row>
+      <xdr:rowOff>42840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3114,15 +3114,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>50800</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1618920</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>18720</xdr:rowOff>
+      <xdr:colOff>1669720</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>488620</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3141,8 +3141,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1618920" cy="447480"/>
+          <a:off x="50800" y="50800"/>
+          <a:ext cx="1618920" cy="437820"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3163,15 +3163,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>50800</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1669720</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>488620</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>581760</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>